<commit_message>
Documente le choix cuivre 1oz et met a jour les fichiers de fab
Garde 1oz (standard) plutot que 2oz (+18$/lot) pour ce proto -
temperature mesuree pendant les tests plutot que supposee, upgrade
possible plus tard si besoin. Fichiers Gerber/BOM/PickAndPlace
regeneres suite au rework du layout (condensateurs electrolytiques
plus gros, plan de masse refait).
</commit_message>
<xml_diff>
--- a/gerber/BOM_Board1_PCB1_2026-07-11.xlsx
+++ b/gerber/BOM_Board1_PCB1_2026-07-11.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_PCB1_2026-07-11" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_PCB1_2026-07-15" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="110">
   <si>
     <t>No.</t>
   </si>
@@ -103,217 +103,232 @@
     <t>5</t>
   </si>
   <si>
-    <t>390µF</t>
+    <t>390uF</t>
   </si>
   <si>
     <t>C9,C14</t>
   </si>
   <si>
+    <t>CAP-SMD_BD10.0-L10.3-W10.3-FD</t>
+  </si>
+  <si>
+    <t>BXJ 35V390 10*10</t>
+  </si>
+  <si>
+    <t>SAMYOUNG(韩国三莹)</t>
+  </si>
+  <si>
+    <t>C359223</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>22uF</t>
+  </si>
+  <si>
+    <t>C10,C12,C13,C15,C18,C20,C21</t>
+  </si>
+  <si>
+    <t>CAP-TH_BD5.0-P2.00-D0.8-FD</t>
+  </si>
+  <si>
+    <t>GR226M050D11RR0VH4FP0</t>
+  </si>
+  <si>
+    <t>Chengx(承兴)</t>
+  </si>
+  <si>
+    <t>C28057</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>1µF</t>
+  </si>
+  <si>
+    <t>C19</t>
+  </si>
+  <si>
     <t>C0603</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>22µF</t>
-  </si>
-  <si>
-    <t>C10,C12,C13,C15,C20,C21</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>C16</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>4,7µF</t>
-  </si>
-  <si>
-    <t>C18</t>
-  </si>
-  <si>
     <t>9</t>
   </si>
   <si>
-    <t>1µF</t>
-  </si>
-  <si>
-    <t>C19</t>
+    <t>DB128L-5.08-4P-GN-S</t>
+  </si>
+  <si>
+    <t>CN1</t>
+  </si>
+  <si>
+    <t>CONN-TH_4P_DB128L-5.08-4P-GN-S</t>
+  </si>
+  <si>
+    <t>DORABO(地博电气)</t>
+  </si>
+  <si>
+    <t>C2827883</t>
   </si>
   <si>
     <t>10</t>
   </si>
   <si>
-    <t>DB128L-5.08-4P-GN-S</t>
-  </si>
-  <si>
-    <t>CN1</t>
-  </si>
-  <si>
-    <t>CONN-TH_4P_DB128L-5.08-4P-GN-S</t>
-  </si>
-  <si>
-    <t>DORABO(地博电气)</t>
-  </si>
-  <si>
-    <t>C2827883</t>
+    <t>MM1Z15</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>SOD-123_L2.8-W1.8-LS3.7-RD</t>
+  </si>
+  <si>
+    <t>晶导微电子</t>
+  </si>
+  <si>
+    <t>C115219</t>
   </si>
   <si>
     <t>11</t>
   </si>
   <si>
-    <t>MM1Z15</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>SOD-123_L2.8-W1.8-LS3.7-RD</t>
-  </si>
-  <si>
-    <t>晶导微电子</t>
-  </si>
-  <si>
-    <t>C115219</t>
+    <t>10uH</t>
+  </si>
+  <si>
+    <t>L1,L2,L3,L4</t>
+  </si>
+  <si>
+    <t>IND-SMD_L7.3-W6.6</t>
+  </si>
+  <si>
+    <t>MHCI06024-100M-R8A</t>
+  </si>
+  <si>
+    <t>Chilisin(奇力新)</t>
+  </si>
+  <si>
+    <t>C280584</t>
   </si>
   <si>
     <t>12</t>
   </si>
   <si>
-    <t>10uH</t>
-  </si>
-  <si>
-    <t>L1,L2,L3,L4</t>
-  </si>
-  <si>
-    <t>IND-SMD_L7.3-W6.6</t>
-  </si>
-  <si>
-    <t>MHCI06024-100M-R8A</t>
-  </si>
-  <si>
-    <t>Chilisin(奇力新)</t>
-  </si>
-  <si>
-    <t>C280584</t>
+    <t>AO4407A</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>SOIC-8_L4.9-W3.9-P1.27-LS6.0-BL</t>
+  </si>
+  <si>
+    <t>AOS</t>
+  </si>
+  <si>
+    <t>C16072</t>
   </si>
   <si>
     <t>13</t>
   </si>
   <si>
-    <t>AO4407A</t>
-  </si>
-  <si>
-    <t>Q1</t>
-  </si>
-  <si>
-    <t>SOIC-8_L4.9-W3.9-P1.27-LS6.0-BL</t>
-  </si>
-  <si>
-    <t>AOS</t>
-  </si>
-  <si>
-    <t>C16072</t>
+    <t>1K</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>R0603</t>
   </si>
   <si>
     <t>14</t>
   </si>
   <si>
-    <t>1K</t>
-  </si>
-  <si>
-    <t>R1</t>
-  </si>
-  <si>
-    <t>R0603</t>
+    <t>15K</t>
+  </si>
+  <si>
+    <t>R2</t>
   </si>
   <si>
     <t>15</t>
   </si>
   <si>
-    <t>15K</t>
-  </si>
-  <si>
-    <t>R2</t>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>R3,R4,R5,R6</t>
   </si>
   <si>
     <t>16</t>
   </si>
   <si>
-    <t>10K</t>
-  </si>
-  <si>
-    <t>R3,R4,R5,R6</t>
+    <t>4.7K</t>
+  </si>
+  <si>
+    <t>R7</t>
   </si>
   <si>
     <t>17</t>
   </si>
   <si>
-    <t>4.7K</t>
-  </si>
-  <si>
-    <t>R7</t>
+    <t>0</t>
+  </si>
+  <si>
+    <t>R8</t>
   </si>
   <si>
     <t>18</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>R8</t>
+    <t>100K</t>
+  </si>
+  <si>
+    <t>R9</t>
   </si>
   <si>
     <t>19</t>
   </si>
   <si>
-    <t>100K</t>
-  </si>
-  <si>
-    <t>R9</t>
+    <t>TAS5825MRHBR</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>VQFN-32_L5.0-W5.0-P0.50-TL-EP</t>
+  </si>
+  <si>
+    <t>TI(德州仪器)</t>
+  </si>
+  <si>
+    <t>C471049</t>
   </si>
   <si>
     <t>20</t>
   </si>
   <si>
-    <t>TAS5825MRHBR</t>
-  </si>
-  <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>VQFN-32_L5.0-W5.0-P0.50-TL-EP</t>
-  </si>
-  <si>
-    <t>TI(德州仪器)</t>
-  </si>
-  <si>
-    <t>C471049</t>
+    <t>B7B-XH-A(LF)(SN)</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>CONN-TH_7P-P2.50_B7B-XH-A-LF-SN</t>
+  </si>
+  <si>
+    <t>JST</t>
+  </si>
+  <si>
+    <t>C144398</t>
   </si>
   <si>
     <t>21</t>
-  </si>
-  <si>
-    <t>B7B-XH-A(LF)(SN)</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>CONN-TH_7P-P2.50_B7B-XH-A-LF-SN</t>
-  </si>
-  <si>
-    <t>JST</t>
-  </si>
-  <si>
-    <t>C144398</t>
-  </si>
-  <si>
-    <t>22</t>
   </si>
   <si>
     <t>DB128L-5.08-2P-GN-S</t>
@@ -702,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -888,53 +903,53 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H6" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="I6" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="J6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G7" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="H7" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="I7" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="J7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -943,7 +958,7 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
         <v>13</v>
@@ -966,22 +981,22 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="G9" t="s">
         <v>16</v>
@@ -998,63 +1013,63 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="H10" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="I10" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="J10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="F11" t="s">
         <v>16</v>
       </c>
       <c r="G11" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="H11" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="I11" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="J11" t="s">
         <v>17</v>
@@ -1062,31 +1077,31 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="G12" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="H12" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="I12" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="J12" t="s">
         <v>17</v>
@@ -1094,31 +1109,31 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="I13" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="J13" t="s">
         <v>17</v>
@@ -1126,54 +1141,54 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="E14" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="F14" t="s">
-        <v>16</v>
+        <v>75</v>
       </c>
       <c r="G14" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="H14" t="s">
-        <v>67</v>
+        <v>16</v>
       </c>
       <c r="I14" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="J14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="D15" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="G15" t="s">
         <v>16</v>
@@ -1190,22 +1205,22 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E16" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="G16" t="s">
         <v>16</v>
@@ -1222,22 +1237,22 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E17" t="s">
         <v>77</v>
       </c>
-      <c r="D17" t="s">
-        <v>78</v>
-      </c>
-      <c r="E17" t="s">
-        <v>72</v>
-      </c>
       <c r="F17" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G17" t="s">
         <v>16</v>
@@ -1254,22 +1269,22 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="D18" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F18" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G18" t="s">
         <v>16</v>
@@ -1286,22 +1301,22 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D19" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E19" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F19" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="G19" t="s">
         <v>16</v>
@@ -1318,63 +1333,63 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D20" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="E20" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="F20" t="s">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="G20" t="s">
-        <v>16</v>
+        <v>94</v>
       </c>
       <c r="H20" t="s">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="I20" t="s">
-        <v>16</v>
+        <v>98</v>
       </c>
       <c r="J20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="D21" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="E21" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="F21" t="s">
         <v>16</v>
       </c>
       <c r="G21" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="H21" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="I21" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="J21" t="s">
         <v>17</v>
@@ -1382,70 +1397,38 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="D22" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E22" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="F22" t="s">
         <v>16</v>
       </c>
       <c r="G22" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="H22" t="s">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="I22" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="J22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>100</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
-        <v>101</v>
-      </c>
-      <c r="D23" t="s">
-        <v>102</v>
-      </c>
-      <c r="E23" t="s">
-        <v>103</v>
-      </c>
-      <c r="F23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" t="s">
-        <v>101</v>
-      </c>
-      <c r="H23" t="s">
-        <v>48</v>
-      </c>
-      <c r="I23" t="s">
-        <v>104</v>
-      </c>
-      <c r="J23" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>